<commit_message>
Actualización de Gantt y Plan de trabajo
</commit_message>
<xml_diff>
--- a/Capstone/Fase 1/Grupales/Plan de trabajo.xlsx
+++ b/Capstone/Fase 1/Grupales/Plan de trabajo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alogo\Desktop\Proyectos\Proyecto-Yourmeds\Capstone\Fase 1\Grupales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CAA477D-C026-4D61-969B-DE54A3279F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4236F1B-C65D-4644-862C-85214AD5D4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nuevo Plan de trabajo" sheetId="1" r:id="rId1"/>
@@ -888,7 +888,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="3" t="s">
@@ -899,7 +899,7 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="3" t="s">
@@ -910,7 +910,7 @@
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="3" t="s">
@@ -921,7 +921,7 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1105,7 +1105,7 @@
         <v>45</v>
       </c>
       <c r="E13" s="10">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F13" s="21" t="s">
         <v>36</v>
@@ -1128,7 +1128,7 @@
         <v>50</v>
       </c>
       <c r="E14" s="10">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F14" s="21" t="s">
         <v>16</v>
@@ -1151,7 +1151,7 @@
         <v>55</v>
       </c>
       <c r="E15" s="10">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F15" s="21" t="s">
         <v>36</v>
@@ -1312,7 +1312,7 @@
         <v>86</v>
       </c>
       <c r="E22" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="23" t="s">
         <v>22</v>
@@ -1335,7 +1335,7 @@
         <v>90</v>
       </c>
       <c r="E23" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" s="23" t="s">
         <v>36</v>

</xml_diff>